<commit_message>
added updated aktiviteter årshjul
</commit_message>
<xml_diff>
--- a/Årshjul for aktiviteter.xlsx
+++ b/Årshjul for aktiviteter.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30317"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/niclasl/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://exactaas-my.sharepoint.com/personal/naja_exacta_no/Documents/Region VV/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{672A6D7A-A76B-5449-9176-C22B45849707}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="250" documentId="8_{E6C819CA-2D33-450E-8E61-5DFE69E49034}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{79F01EF2-0971-4F9E-BC1C-A10AFBC2AB4D}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="520" windowWidth="26240" windowHeight="16440" firstSheet="1" activeTab="1" xr2:uid="{784348BC-1604-447D-9126-6798E5DC6166}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{784348BC-1604-447D-9126-6798E5DC6166}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="89">
   <si>
     <t>Antall aktiviteter</t>
   </si>
@@ -287,28 +287,13 @@
     <t>46275 – Aktivitet 9 (Naja)</t>
   </si>
   <si>
-    <t>Regionsturnering U15</t>
-  </si>
-  <si>
     <t>46285 – Aktivitet 8 (Magnus)</t>
   </si>
   <si>
-    <t>Mesterskap JU14</t>
-  </si>
-  <si>
     <t>46295 – Aktivitet 7 (Naja)</t>
   </si>
   <si>
-    <t>Mesterskap U14</t>
-  </si>
-  <si>
-    <t>Bærum Ishall</t>
-  </si>
-  <si>
     <t>46305 – Aktivitet 6 (Magnus)</t>
-  </si>
-  <si>
-    <t>RegionsturneringJU16</t>
   </si>
   <si>
     <t>46315 – Aktivitet 5 (Naja)</t>
@@ -333,7 +318,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/m/;@"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1199,8 +1184,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="12947651" y="292100"/>
-              <a:ext cx="12874624" cy="6235700"/>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -1219,9 +1204,9 @@
             <a:lstStyle/>
             <a:p>
               <a:r>
-                <a:rPr lang="en-US" sz="1100"/>
-                <a:t>This chart isn't available in your version of Excel.
-Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+                <a:rPr sz="1100"/>
+                <a:t>Dette diagrammet er ikke tilgjengelig i din versjon av Excel.
+Hvis du redigerer denne figuren eller lagrer denne arbeidsboken i et annet filformat, blir diagrammet ødelagt for godt.</a:t>
               </a:r>
             </a:p>
           </xdr:txBody>
@@ -1578,39 +1563,17 @@
 </a:theme>
 </file>
 
-<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
-<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </wetp:taskpane>
-</wetp:taskpanes>
-</file>
-
-<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{6BE9EE7C-E41D-6C44-AE42-98DC36BE8E4A}">
-  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
-  <we:alternateReferences>
-    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
-  </we:alternateReferences>
-  <we:properties>
-    <we:property name="claude.fileId" value="&quot;d76187fb-57ab-4f1c-be68-89011a9555d2&quot;"/>
-  </we:properties>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</we:webextension>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B929DAC1-2435-45A8-877C-8697E4CDC1B7}">
   <dimension ref="A2:D30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1624,7 +1587,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -1638,7 +1601,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -1652,7 +1615,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -1666,7 +1629,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -1680,7 +1643,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4">
       <c r="A8" s="1" t="s">
         <v>12</v>
       </c>
@@ -1694,7 +1657,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
@@ -1708,7 +1671,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -1722,7 +1685,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4">
       <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
@@ -1736,7 +1699,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4">
       <c r="A12" s="1" t="s">
         <v>16</v>
       </c>
@@ -1750,7 +1713,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4">
       <c r="A13" s="1" t="s">
         <v>20</v>
       </c>
@@ -1764,7 +1727,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -1778,7 +1741,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4">
       <c r="A15" s="1" t="s">
         <v>23</v>
       </c>
@@ -1792,7 +1755,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4">
       <c r="A16" s="1" t="s">
         <v>25</v>
       </c>
@@ -1806,7 +1769,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4">
       <c r="A17" s="1" t="s">
         <v>27</v>
       </c>
@@ -1820,7 +1783,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4">
       <c r="A18" s="1" t="s">
         <v>27</v>
       </c>
@@ -1834,7 +1797,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4">
       <c r="A19" s="1" t="s">
         <v>30</v>
       </c>
@@ -1848,7 +1811,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4">
       <c r="A20" s="1" t="s">
         <v>30</v>
       </c>
@@ -1862,7 +1825,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4">
       <c r="A21" s="1" t="s">
         <v>30</v>
       </c>
@@ -1876,7 +1839,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4">
       <c r="A22" s="1" t="s">
         <v>30</v>
       </c>
@@ -1890,7 +1853,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4">
       <c r="A23" s="1" t="s">
         <v>35</v>
       </c>
@@ -1904,7 +1867,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4">
       <c r="A24" s="1" t="s">
         <v>35</v>
       </c>
@@ -1918,7 +1881,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4">
       <c r="A25" s="1" t="s">
         <v>35</v>
       </c>
@@ -1932,7 +1895,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4">
       <c r="A26" s="1" t="s">
         <v>39</v>
       </c>
@@ -1946,7 +1909,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4">
       <c r="A27" s="1" t="s">
         <v>39</v>
       </c>
@@ -1960,7 +1923,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4">
       <c r="A28" s="1" t="s">
         <v>39</v>
       </c>
@@ -1974,7 +1937,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4">
       <c r="A29" s="1" t="s">
         <v>43</v>
       </c>
@@ -1988,7 +1951,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4">
       <c r="A30" s="1" t="s">
         <v>43</v>
       </c>
@@ -2009,22 +1972,22 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6E61283-F91B-45F4-8D2D-0D7683221028}">
-  <dimension ref="A1:N41"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:N120"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="0.5" customWidth="1"/>
-    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="0.5703125" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="6" max="6" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.1640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.42578125" bestFit="1" customWidth="1"/>
     <col min="13" max="14" width="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="22" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="21">
       <c r="A1" s="6" t="s">
         <v>46</v>
       </c>
@@ -2036,7 +1999,7 @@
       <c r="G1" s="7"/>
       <c r="H1" s="7"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
         <v>47</v>
       </c>
@@ -2071,7 +2034,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14">
       <c r="A4">
         <v>1</v>
       </c>
@@ -2104,7 +2067,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14">
       <c r="A5">
         <v>1</v>
       </c>
@@ -2137,7 +2100,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14">
       <c r="A6">
         <v>2</v>
       </c>
@@ -2170,7 +2133,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14">
       <c r="A7">
         <v>2</v>
       </c>
@@ -2203,7 +2166,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14">
       <c r="A8">
         <v>2</v>
       </c>
@@ -2236,7 +2199,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14">
       <c r="A9">
         <v>3</v>
       </c>
@@ -2269,7 +2232,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14">
       <c r="A10">
         <v>3</v>
       </c>
@@ -2302,7 +2265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14">
       <c r="A11">
         <v>3</v>
       </c>
@@ -2338,7 +2301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14">
       <c r="A12">
         <v>4</v>
       </c>
@@ -2374,7 +2337,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14">
       <c r="A13">
         <v>4</v>
       </c>
@@ -2410,7 +2373,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14">
       <c r="A14">
         <v>4</v>
       </c>
@@ -2446,7 +2409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14">
       <c r="A15">
         <v>4</v>
       </c>
@@ -2482,7 +2445,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14">
       <c r="A16">
         <v>5</v>
       </c>
@@ -2511,7 +2474,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:14">
       <c r="A17">
         <v>5</v>
       </c>
@@ -2537,7 +2500,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:14">
       <c r="A18">
         <v>6</v>
       </c>
@@ -2563,7 +2526,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:14" ht="15">
       <c r="A19">
         <v>7</v>
       </c>
@@ -2589,7 +2552,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:14" ht="15">
       <c r="A20">
         <v>8</v>
       </c>
@@ -2615,7 +2578,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:14" ht="15">
       <c r="A21">
         <v>8</v>
       </c>
@@ -2641,7 +2604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:14" ht="15">
       <c r="A22">
         <v>9</v>
       </c>
@@ -2660,14 +2623,11 @@
       <c r="K22" s="9">
         <v>46136</v>
       </c>
-      <c r="L22" t="s">
-        <v>81</v>
-      </c>
       <c r="N22" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:14" ht="15">
       <c r="A23">
         <v>9</v>
       </c>
@@ -2675,7 +2635,7 @@
         <v>16</v>
       </c>
       <c r="C23" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -2686,14 +2646,11 @@
       <c r="K23" s="9">
         <v>46130</v>
       </c>
-      <c r="L23" t="s">
-        <v>83</v>
-      </c>
       <c r="N23" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:14" ht="15">
       <c r="A24">
         <v>9</v>
       </c>
@@ -2701,7 +2658,7 @@
         <v>16</v>
       </c>
       <c r="C24" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -2712,17 +2669,11 @@
       <c r="K24" s="9">
         <v>46129</v>
       </c>
-      <c r="L24" t="s">
-        <v>85</v>
-      </c>
-      <c r="M24" t="s">
-        <v>86</v>
-      </c>
       <c r="N24" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:14" ht="15">
       <c r="A25">
         <v>10</v>
       </c>
@@ -2730,7 +2681,7 @@
         <v>12</v>
       </c>
       <c r="C25" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D25">
         <v>1</v>
@@ -2741,14 +2692,11 @@
       <c r="K25" s="9">
         <v>46122</v>
       </c>
-      <c r="L25" t="s">
-        <v>88</v>
-      </c>
       <c r="N25" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:14" ht="15">
       <c r="A26">
         <v>10</v>
       </c>
@@ -2756,7 +2704,7 @@
         <v>12</v>
       </c>
       <c r="C26" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D26">
         <v>1</v>
@@ -2774,7 +2722,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:14" ht="15">
       <c r="A27">
         <v>10</v>
       </c>
@@ -2782,7 +2730,7 @@
         <v>12</v>
       </c>
       <c r="C27" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -2800,7 +2748,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:14" ht="15">
       <c r="A28">
         <v>11</v>
       </c>
@@ -2808,7 +2756,7 @@
         <v>8</v>
       </c>
       <c r="C28" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="D28">
         <v>1</v>
@@ -2826,7 +2774,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:14" ht="15">
       <c r="A29">
         <v>11</v>
       </c>
@@ -2834,7 +2782,7 @@
         <v>8</v>
       </c>
       <c r="C29" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="D29">
         <v>1</v>
@@ -2852,7 +2800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:14" ht="15">
       <c r="A30">
         <v>12</v>
       </c>
@@ -2860,7 +2808,7 @@
         <v>5</v>
       </c>
       <c r="C30" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D30">
         <v>1</v>
@@ -2878,7 +2826,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:14" ht="15">
       <c r="J31" t="s">
         <v>39</v>
       </c>
@@ -2892,7 +2840,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:14" ht="15">
       <c r="J32" t="s">
         <v>39</v>
       </c>
@@ -2906,7 +2854,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="33" spans="10:14" ht="15">
       <c r="J33" t="s">
         <v>39</v>
       </c>
@@ -2920,7 +2868,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="34" spans="10:14" ht="15">
       <c r="J34" t="s">
         <v>43</v>
       </c>
@@ -2934,7 +2882,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="35" spans="10:14" ht="15">
       <c r="J35" t="s">
         <v>43</v>
       </c>
@@ -2948,30 +2896,109 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="36" spans="10:14" ht="15">
       <c r="K36" s="9"/>
       <c r="N36" s="5"/>
     </row>
-    <row r="37" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="37" spans="10:14" ht="15">
       <c r="K37" s="9"/>
       <c r="N37" s="5"/>
     </row>
-    <row r="38" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="38" spans="10:14" ht="15">
       <c r="K38" s="9"/>
       <c r="N38" s="5"/>
     </row>
-    <row r="39" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="39" spans="10:14" ht="15">
       <c r="K39" s="9"/>
       <c r="N39" s="5"/>
     </row>
-    <row r="40" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="40" spans="10:14" ht="15">
       <c r="K40" s="9"/>
       <c r="N40" s="5"/>
     </row>
-    <row r="41" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="41" spans="10:14" ht="15">
       <c r="K41" s="9"/>
       <c r="N41" s="5"/>
     </row>
+    <row r="42" spans="10:14" ht="15"/>
+    <row r="43" spans="10:14" ht="15"/>
+    <row r="44" spans="10:14" ht="15"/>
+    <row r="45" spans="10:14" ht="15"/>
+    <row r="46" spans="10:14" ht="15"/>
+    <row r="47" spans="10:14" ht="15"/>
+    <row r="48" spans="10:14" ht="15"/>
+    <row r="49" ht="15"/>
+    <row r="50" ht="15"/>
+    <row r="51" ht="15"/>
+    <row r="52" ht="15"/>
+    <row r="53" ht="15"/>
+    <row r="54" ht="15"/>
+    <row r="55" ht="15"/>
+    <row r="56" ht="15"/>
+    <row r="57" ht="15"/>
+    <row r="58" ht="15"/>
+    <row r="59" ht="15"/>
+    <row r="60" ht="15"/>
+    <row r="61" ht="15"/>
+    <row r="62" ht="15"/>
+    <row r="63" ht="15"/>
+    <row r="64" ht="15"/>
+    <row r="65" ht="15"/>
+    <row r="66" ht="15"/>
+    <row r="67" ht="15"/>
+    <row r="68" ht="15"/>
+    <row r="69" ht="15"/>
+    <row r="70" ht="15"/>
+    <row r="71" ht="15"/>
+    <row r="72" ht="15"/>
+    <row r="73" ht="15"/>
+    <row r="74" ht="15"/>
+    <row r="75" ht="15"/>
+    <row r="76" ht="15"/>
+    <row r="77" ht="15"/>
+    <row r="78" ht="15"/>
+    <row r="79" ht="15"/>
+    <row r="80" ht="15"/>
+    <row r="81" ht="15"/>
+    <row r="82" ht="15"/>
+    <row r="83" ht="15"/>
+    <row r="84" ht="15"/>
+    <row r="85" ht="15"/>
+    <row r="86" ht="15"/>
+    <row r="87" ht="15"/>
+    <row r="88" ht="15"/>
+    <row r="89" ht="15"/>
+    <row r="90" ht="15"/>
+    <row r="91" ht="15"/>
+    <row r="92" ht="15"/>
+    <row r="93" ht="15"/>
+    <row r="94" ht="15"/>
+    <row r="95" ht="15"/>
+    <row r="96" ht="15"/>
+    <row r="97" ht="15"/>
+    <row r="98" ht="15"/>
+    <row r="99" ht="15"/>
+    <row r="100" ht="15"/>
+    <row r="101" ht="15"/>
+    <row r="102" ht="15"/>
+    <row r="103" ht="15"/>
+    <row r="104" ht="15"/>
+    <row r="105" ht="15"/>
+    <row r="106" ht="15"/>
+    <row r="107" ht="15"/>
+    <row r="108" ht="15"/>
+    <row r="109" ht="15"/>
+    <row r="110" ht="15"/>
+    <row r="111" ht="15"/>
+    <row r="112" ht="15"/>
+    <row r="113" ht="15"/>
+    <row r="114" ht="15"/>
+    <row r="115" ht="15"/>
+    <row r="116" ht="15"/>
+    <row r="117" ht="15"/>
+    <row r="118" ht="15"/>
+    <row r="119" ht="15"/>
+    <row r="120" ht="15"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2983,21 +3010,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100F2DFD330500C9D4C80E12BEFCF165AD3" ma:contentTypeVersion="8" ma:contentTypeDescription="Opprett et nytt dokument." ma:contentTypeScope="" ma:versionID="393035f51cba4c419aa8a34d1a6c616e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ba88375d-8b29-4298-897f-8fd300d2f4ef" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="04bc00d8e9204182f4d597b94839611d" ns2:_="">
     <xsd:import namespace="ba88375d-8b29-4298-897f-8fd300d2f4ef"/>
@@ -3167,37 +3179,29 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{773E4754-7A49-4480-A992-A2E42BA68227}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4B9B597-C5DB-42F8-8050-887D65052BF6}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F1C20245-DDC0-4D79-9C7A-D3560D80B718}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{773E4754-7A49-4480-A992-A2E42BA68227}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4B9B597-C5DB-42F8-8050-887D65052BF6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="ba88375d-8b29-4298-897f-8fd300d2f4ef"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F1C20245-DDC0-4D79-9C7A-D3560D80B718}"/>
 </file>
</xml_diff>